<commit_message>
data collection for experiment 2
</commit_message>
<xml_diff>
--- a/Experiment 2 - Comparing Diffusion to Chemotaxis/Time_for_Bac_Fix_Comparison.xlsx
+++ b/Experiment 2 - Comparing Diffusion to Chemotaxis/Time_for_Bac_Fix_Comparison.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Moar Documents\GitHub\Bac_Evol_SSA\Experiment 2 - Comparing Diffusion to Chemotaxis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90FA7E43-7A0C-435B-AAED-42CFFF793DA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{537E53E5-C3A2-415B-A65C-0C224D65D57C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9120" yWindow="1605" windowWidth="18675" windowHeight="12975" xr2:uid="{C5D5DF43-D68A-448F-BEE9-BC751A2734F3}"/>
+    <workbookView xWindow="9555" yWindow="1860" windowWidth="18675" windowHeight="12975" xr2:uid="{C5D5DF43-D68A-448F-BEE9-BC751A2734F3}"/>
   </bookViews>
   <sheets>
     <sheet name="All Time Distributions" sheetId="2" r:id="rId1"/>
@@ -503,346 +503,538 @@
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>19232</v>
+      </c>
       <c r="B12">
         <v>30543</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>11287</v>
+      </c>
       <c r="B13">
         <v>29016</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>21931</v>
+      </c>
       <c r="B14">
         <v>22487</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>19650</v>
+      </c>
       <c r="B15">
         <v>22189</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>26696</v>
+      </c>
       <c r="B16">
         <v>21234</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>17714</v>
+      </c>
       <c r="B17">
         <v>24318</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>25094</v>
+      </c>
       <c r="B18">
         <v>22289</v>
       </c>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>28007</v>
+      </c>
       <c r="B19">
         <v>25336</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>18679</v>
+      </c>
       <c r="B20">
         <v>25372</v>
       </c>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>19643</v>
+      </c>
       <c r="B21">
         <v>19683</v>
       </c>
     </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21265</v>
+      </c>
       <c r="B22">
         <v>25776</v>
       </c>
     </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>21377</v>
+      </c>
       <c r="B23">
         <v>26909</v>
       </c>
     </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>22322</v>
+      </c>
       <c r="B24">
         <v>28253</v>
       </c>
     </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24275</v>
+      </c>
       <c r="B25">
         <v>27650</v>
       </c>
     </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>30816</v>
+      </c>
       <c r="B26">
         <v>26881</v>
       </c>
     </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>16545</v>
+      </c>
       <c r="B27">
         <v>10800</v>
       </c>
     </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>19903</v>
+      </c>
       <c r="B28">
         <v>24028</v>
       </c>
     </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>39176</v>
+      </c>
       <c r="B29">
         <v>32241</v>
       </c>
     </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>21530</v>
+      </c>
       <c r="B30">
         <v>27336</v>
       </c>
     </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>21976</v>
+      </c>
       <c r="B31">
         <v>26020</v>
       </c>
     </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>24713</v>
+      </c>
       <c r="B32">
         <v>27785</v>
       </c>
     </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>23243</v>
+      </c>
       <c r="B33">
         <v>36116</v>
       </c>
     </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>21561</v>
+      </c>
       <c r="B34">
         <v>23131</v>
       </c>
     </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>21740</v>
+      </c>
       <c r="B35">
         <v>23689</v>
       </c>
     </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>18463</v>
+      </c>
       <c r="B36">
         <v>25583</v>
       </c>
     </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>17179</v>
+      </c>
       <c r="B37">
         <v>26749</v>
       </c>
     </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>24412</v>
+      </c>
       <c r="B38">
         <v>21655</v>
       </c>
     </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>26431</v>
+      </c>
       <c r="B39">
         <v>6792</v>
       </c>
     </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>23323</v>
+      </c>
       <c r="B40">
         <v>26589</v>
       </c>
     </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>26872</v>
+      </c>
       <c r="B41">
         <v>24613</v>
       </c>
     </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>19027</v>
+      </c>
       <c r="B42">
         <v>24126</v>
       </c>
     </row>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>28879</v>
+      </c>
       <c r="B43">
         <v>22769</v>
       </c>
     </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>18884</v>
+      </c>
       <c r="B44">
         <v>34003</v>
       </c>
     </row>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>20187</v>
+      </c>
       <c r="B45">
         <v>23840</v>
       </c>
     </row>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>36209</v>
+      </c>
       <c r="B46">
         <v>24015</v>
       </c>
     </row>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>21322</v>
+      </c>
       <c r="B47">
         <v>27152</v>
       </c>
     </row>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>26316</v>
+      </c>
       <c r="B48">
         <v>24951</v>
       </c>
     </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>19711</v>
+      </c>
       <c r="B49">
         <v>22722</v>
       </c>
     </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>24521</v>
+      </c>
       <c r="B50">
         <v>25137</v>
       </c>
     </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>28146</v>
+      </c>
       <c r="B51">
         <v>23155</v>
       </c>
     </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>18798</v>
+      </c>
       <c r="B52">
         <v>23006</v>
       </c>
     </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>28569</v>
+      </c>
       <c r="B53">
         <v>27796</v>
       </c>
     </row>
-    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>25077</v>
+      </c>
       <c r="B54">
         <v>29204</v>
       </c>
     </row>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>29094</v>
+      </c>
       <c r="B55">
         <v>28927</v>
       </c>
     </row>
-    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>24085</v>
+      </c>
       <c r="B56">
         <v>22924</v>
       </c>
     </row>
-    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>19852</v>
+      </c>
       <c r="B57">
         <v>33235</v>
       </c>
     </row>
-    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>21048</v>
+      </c>
       <c r="B58">
         <v>22867</v>
       </c>
     </row>
-    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>17948</v>
+      </c>
       <c r="B59">
         <v>20071</v>
       </c>
     </row>
-    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>16730</v>
+      </c>
       <c r="B60">
         <v>21999</v>
       </c>
     </row>
-    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>22241</v>
+      </c>
       <c r="B61">
         <v>34240</v>
       </c>
     </row>
-    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>12174</v>
+      </c>
       <c r="B62">
         <v>29276</v>
       </c>
     </row>
-    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>28310</v>
+      </c>
       <c r="B63">
         <v>31260</v>
       </c>
     </row>
-    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>19955</v>
+      </c>
       <c r="B64">
         <v>27076</v>
       </c>
     </row>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>22235</v>
+      </c>
       <c r="B65">
         <v>18543</v>
       </c>
     </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>18482</v>
+      </c>
       <c r="B66">
         <v>28416</v>
       </c>
     </row>
-    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>16728</v>
+      </c>
       <c r="B67">
         <v>25600</v>
       </c>
     </row>
-    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>13341</v>
+      </c>
       <c r="B68">
         <v>32846</v>
       </c>
     </row>
-    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>20871</v>
+      </c>
       <c r="B69">
         <v>22337</v>
       </c>
     </row>
-    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>29148</v>
+      </c>
       <c r="B70">
         <v>23836</v>
       </c>
     </row>
-    <row r="71" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>19996</v>
+      </c>
       <c r="B71">
         <v>24079</v>
       </c>
     </row>
-    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>21397</v>
+      </c>
       <c r="B72">
         <v>20540</v>
       </c>
     </row>
-    <row r="73" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>19346</v>
+      </c>
       <c r="B73">
         <v>26668</v>
       </c>
     </row>
-    <row r="74" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>24691</v>
+      </c>
       <c r="B74">
         <v>22659</v>
       </c>
     </row>
-    <row r="75" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>20727</v>
+      </c>
       <c r="B75">
         <v>31241</v>
       </c>
     </row>
-    <row r="76" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B76">
         <v>21113</v>
       </c>
     </row>
-    <row r="77" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B77">
         <v>25566</v>
       </c>
     </row>
-    <row r="78" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B78">
         <v>23726</v>
       </c>
     </row>
-    <row r="79" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B79">
         <v>36392</v>
       </c>
     </row>
-    <row r="80" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B80">
         <v>16003</v>
       </c>
@@ -959,7 +1151,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14A4F54D-F9A8-4A57-B36F-2ADC46C86094}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
@@ -1085,6 +1277,838 @@
       </c>
       <c r="C11">
         <v>5.4563888888888892</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>19232</v>
+      </c>
+      <c r="B12">
+        <f>A12/60</f>
+        <v>320.53333333333336</v>
+      </c>
+      <c r="C12">
+        <f>A12/3600</f>
+        <v>5.3422222222222224</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>11287</v>
+      </c>
+      <c r="B13">
+        <f t="shared" ref="B13:B75" si="0">A13/60</f>
+        <v>188.11666666666667</v>
+      </c>
+      <c r="C13">
+        <f t="shared" ref="C13:C75" si="1">A13/3600</f>
+        <v>3.1352777777777776</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>21931</v>
+      </c>
+      <c r="B14">
+        <f t="shared" si="0"/>
+        <v>365.51666666666665</v>
+      </c>
+      <c r="C14">
+        <f t="shared" si="1"/>
+        <v>6.0919444444444446</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>19650</v>
+      </c>
+      <c r="B15">
+        <f t="shared" si="0"/>
+        <v>327.5</v>
+      </c>
+      <c r="C15">
+        <f t="shared" si="1"/>
+        <v>5.458333333333333</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>26696</v>
+      </c>
+      <c r="B16">
+        <f t="shared" si="0"/>
+        <v>444.93333333333334</v>
+      </c>
+      <c r="C16">
+        <f t="shared" si="1"/>
+        <v>7.4155555555555557</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>17714</v>
+      </c>
+      <c r="B17">
+        <f t="shared" si="0"/>
+        <v>295.23333333333335</v>
+      </c>
+      <c r="C17">
+        <f t="shared" si="1"/>
+        <v>4.9205555555555556</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>25094</v>
+      </c>
+      <c r="B18">
+        <f t="shared" si="0"/>
+        <v>418.23333333333335</v>
+      </c>
+      <c r="C18">
+        <f t="shared" si="1"/>
+        <v>6.9705555555555554</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>28007</v>
+      </c>
+      <c r="B19">
+        <f t="shared" si="0"/>
+        <v>466.78333333333336</v>
+      </c>
+      <c r="C19">
+        <f t="shared" si="1"/>
+        <v>7.7797222222222224</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>18679</v>
+      </c>
+      <c r="B20">
+        <f t="shared" si="0"/>
+        <v>311.31666666666666</v>
+      </c>
+      <c r="C20">
+        <f t="shared" si="1"/>
+        <v>5.1886111111111113</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>19643</v>
+      </c>
+      <c r="B21">
+        <f t="shared" si="0"/>
+        <v>327.38333333333333</v>
+      </c>
+      <c r="C21">
+        <f t="shared" si="1"/>
+        <v>5.4563888888888892</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21265</v>
+      </c>
+      <c r="B22">
+        <f t="shared" si="0"/>
+        <v>354.41666666666669</v>
+      </c>
+      <c r="C22">
+        <f t="shared" si="1"/>
+        <v>5.9069444444444441</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>21377</v>
+      </c>
+      <c r="B23">
+        <f t="shared" si="0"/>
+        <v>356.28333333333336</v>
+      </c>
+      <c r="C23">
+        <f t="shared" si="1"/>
+        <v>5.9380555555555556</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>22322</v>
+      </c>
+      <c r="B24">
+        <f t="shared" si="0"/>
+        <v>372.03333333333336</v>
+      </c>
+      <c r="C24">
+        <f t="shared" si="1"/>
+        <v>6.2005555555555558</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24275</v>
+      </c>
+      <c r="B25">
+        <f t="shared" si="0"/>
+        <v>404.58333333333331</v>
+      </c>
+      <c r="C25">
+        <f t="shared" si="1"/>
+        <v>6.7430555555555554</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>30816</v>
+      </c>
+      <c r="B26">
+        <f t="shared" si="0"/>
+        <v>513.6</v>
+      </c>
+      <c r="C26">
+        <f t="shared" si="1"/>
+        <v>8.56</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>16545</v>
+      </c>
+      <c r="B27">
+        <f t="shared" si="0"/>
+        <v>275.75</v>
+      </c>
+      <c r="C27">
+        <f t="shared" si="1"/>
+        <v>4.5958333333333332</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>19903</v>
+      </c>
+      <c r="B28">
+        <f t="shared" si="0"/>
+        <v>331.71666666666664</v>
+      </c>
+      <c r="C28">
+        <f t="shared" si="1"/>
+        <v>5.5286111111111111</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>39176</v>
+      </c>
+      <c r="B29">
+        <f t="shared" si="0"/>
+        <v>652.93333333333328</v>
+      </c>
+      <c r="C29">
+        <f t="shared" si="1"/>
+        <v>10.882222222222222</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>21530</v>
+      </c>
+      <c r="B30">
+        <f t="shared" si="0"/>
+        <v>358.83333333333331</v>
+      </c>
+      <c r="C30">
+        <f t="shared" si="1"/>
+        <v>5.9805555555555552</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>21976</v>
+      </c>
+      <c r="B31">
+        <f t="shared" si="0"/>
+        <v>366.26666666666665</v>
+      </c>
+      <c r="C31">
+        <f t="shared" si="1"/>
+        <v>6.1044444444444448</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>24713</v>
+      </c>
+      <c r="B32">
+        <f t="shared" si="0"/>
+        <v>411.88333333333333</v>
+      </c>
+      <c r="C32">
+        <f t="shared" si="1"/>
+        <v>6.8647222222222224</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>23243</v>
+      </c>
+      <c r="B33">
+        <f t="shared" si="0"/>
+        <v>387.38333333333333</v>
+      </c>
+      <c r="C33">
+        <f t="shared" si="1"/>
+        <v>6.4563888888888892</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>21561</v>
+      </c>
+      <c r="B34">
+        <f t="shared" si="0"/>
+        <v>359.35</v>
+      </c>
+      <c r="C34">
+        <f t="shared" si="1"/>
+        <v>5.9891666666666667</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>21740</v>
+      </c>
+      <c r="B35">
+        <f t="shared" si="0"/>
+        <v>362.33333333333331</v>
+      </c>
+      <c r="C35">
+        <f t="shared" si="1"/>
+        <v>6.0388888888888888</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>18463</v>
+      </c>
+      <c r="B36">
+        <f t="shared" si="0"/>
+        <v>307.71666666666664</v>
+      </c>
+      <c r="C36">
+        <f t="shared" si="1"/>
+        <v>5.1286111111111108</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>17179</v>
+      </c>
+      <c r="B37">
+        <f t="shared" si="0"/>
+        <v>286.31666666666666</v>
+      </c>
+      <c r="C37">
+        <f t="shared" si="1"/>
+        <v>4.7719444444444443</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>24412</v>
+      </c>
+      <c r="B38">
+        <f t="shared" si="0"/>
+        <v>406.86666666666667</v>
+      </c>
+      <c r="C38">
+        <f t="shared" si="1"/>
+        <v>6.7811111111111115</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>26431</v>
+      </c>
+      <c r="B39">
+        <f t="shared" si="0"/>
+        <v>440.51666666666665</v>
+      </c>
+      <c r="C39">
+        <f t="shared" si="1"/>
+        <v>7.3419444444444446</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>23323</v>
+      </c>
+      <c r="B40">
+        <f t="shared" si="0"/>
+        <v>388.71666666666664</v>
+      </c>
+      <c r="C40">
+        <f t="shared" si="1"/>
+        <v>6.4786111111111113</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>26872</v>
+      </c>
+      <c r="B41">
+        <f t="shared" si="0"/>
+        <v>447.86666666666667</v>
+      </c>
+      <c r="C41">
+        <f t="shared" si="1"/>
+        <v>7.4644444444444442</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>19027</v>
+      </c>
+      <c r="B42">
+        <f t="shared" si="0"/>
+        <v>317.11666666666667</v>
+      </c>
+      <c r="C42">
+        <f t="shared" si="1"/>
+        <v>5.285277777777778</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>28879</v>
+      </c>
+      <c r="B43">
+        <f t="shared" si="0"/>
+        <v>481.31666666666666</v>
+      </c>
+      <c r="C43">
+        <f t="shared" si="1"/>
+        <v>8.0219444444444452</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>18884</v>
+      </c>
+      <c r="B44">
+        <f t="shared" si="0"/>
+        <v>314.73333333333335</v>
+      </c>
+      <c r="C44">
+        <f t="shared" si="1"/>
+        <v>5.2455555555555557</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>20187</v>
+      </c>
+      <c r="B45">
+        <f t="shared" si="0"/>
+        <v>336.45</v>
+      </c>
+      <c r="C45">
+        <f t="shared" si="1"/>
+        <v>5.6074999999999999</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>36209</v>
+      </c>
+      <c r="B46">
+        <f t="shared" si="0"/>
+        <v>603.48333333333335</v>
+      </c>
+      <c r="C46">
+        <f t="shared" si="1"/>
+        <v>10.058055555555555</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>21322</v>
+      </c>
+      <c r="B47">
+        <f t="shared" si="0"/>
+        <v>355.36666666666667</v>
+      </c>
+      <c r="C47">
+        <f t="shared" si="1"/>
+        <v>5.9227777777777781</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>26316</v>
+      </c>
+      <c r="B48">
+        <f t="shared" si="0"/>
+        <v>438.6</v>
+      </c>
+      <c r="C48">
+        <f t="shared" si="1"/>
+        <v>7.31</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>19711</v>
+      </c>
+      <c r="B49">
+        <f t="shared" si="0"/>
+        <v>328.51666666666665</v>
+      </c>
+      <c r="C49">
+        <f t="shared" si="1"/>
+        <v>5.4752777777777775</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>24521</v>
+      </c>
+      <c r="B50">
+        <f t="shared" si="0"/>
+        <v>408.68333333333334</v>
+      </c>
+      <c r="C50">
+        <f t="shared" si="1"/>
+        <v>6.8113888888888887</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>28146</v>
+      </c>
+      <c r="B51">
+        <f t="shared" si="0"/>
+        <v>469.1</v>
+      </c>
+      <c r="C51">
+        <f t="shared" si="1"/>
+        <v>7.8183333333333334</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>18798</v>
+      </c>
+      <c r="B52">
+        <f t="shared" si="0"/>
+        <v>313.3</v>
+      </c>
+      <c r="C52">
+        <f t="shared" si="1"/>
+        <v>5.2216666666666667</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>28569</v>
+      </c>
+      <c r="B53">
+        <f t="shared" si="0"/>
+        <v>476.15</v>
+      </c>
+      <c r="C53">
+        <f t="shared" si="1"/>
+        <v>7.9358333333333331</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>25077</v>
+      </c>
+      <c r="B54">
+        <f t="shared" si="0"/>
+        <v>417.95</v>
+      </c>
+      <c r="C54">
+        <f t="shared" si="1"/>
+        <v>6.9658333333333333</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>29094</v>
+      </c>
+      <c r="B55">
+        <f t="shared" si="0"/>
+        <v>484.9</v>
+      </c>
+      <c r="C55">
+        <f t="shared" si="1"/>
+        <v>8.081666666666667</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>24085</v>
+      </c>
+      <c r="B56">
+        <f t="shared" si="0"/>
+        <v>401.41666666666669</v>
+      </c>
+      <c r="C56">
+        <f t="shared" si="1"/>
+        <v>6.6902777777777782</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>19852</v>
+      </c>
+      <c r="B57">
+        <f t="shared" si="0"/>
+        <v>330.86666666666667</v>
+      </c>
+      <c r="C57">
+        <f t="shared" si="1"/>
+        <v>5.514444444444444</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>21048</v>
+      </c>
+      <c r="B58">
+        <f t="shared" si="0"/>
+        <v>350.8</v>
+      </c>
+      <c r="C58">
+        <f t="shared" si="1"/>
+        <v>5.8466666666666667</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>17948</v>
+      </c>
+      <c r="B59">
+        <f t="shared" si="0"/>
+        <v>299.13333333333333</v>
+      </c>
+      <c r="C59">
+        <f t="shared" si="1"/>
+        <v>4.985555555555556</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>16730</v>
+      </c>
+      <c r="B60">
+        <f t="shared" si="0"/>
+        <v>278.83333333333331</v>
+      </c>
+      <c r="C60">
+        <f t="shared" si="1"/>
+        <v>4.6472222222222221</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>22241</v>
+      </c>
+      <c r="B61">
+        <f t="shared" si="0"/>
+        <v>370.68333333333334</v>
+      </c>
+      <c r="C61">
+        <f t="shared" si="1"/>
+        <v>6.1780555555555559</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>12174</v>
+      </c>
+      <c r="B62">
+        <f t="shared" si="0"/>
+        <v>202.9</v>
+      </c>
+      <c r="C62">
+        <f t="shared" si="1"/>
+        <v>3.3816666666666668</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>28310</v>
+      </c>
+      <c r="B63">
+        <f t="shared" si="0"/>
+        <v>471.83333333333331</v>
+      </c>
+      <c r="C63">
+        <f t="shared" si="1"/>
+        <v>7.8638888888888889</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>19955</v>
+      </c>
+      <c r="B64">
+        <f t="shared" si="0"/>
+        <v>332.58333333333331</v>
+      </c>
+      <c r="C64">
+        <f t="shared" si="1"/>
+        <v>5.5430555555555552</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>22235</v>
+      </c>
+      <c r="B65">
+        <f t="shared" si="0"/>
+        <v>370.58333333333331</v>
+      </c>
+      <c r="C65">
+        <f t="shared" si="1"/>
+        <v>6.1763888888888889</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>18482</v>
+      </c>
+      <c r="B66">
+        <f t="shared" si="0"/>
+        <v>308.03333333333336</v>
+      </c>
+      <c r="C66">
+        <f t="shared" si="1"/>
+        <v>5.1338888888888885</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>16728</v>
+      </c>
+      <c r="B67">
+        <f t="shared" si="0"/>
+        <v>278.8</v>
+      </c>
+      <c r="C67">
+        <f t="shared" si="1"/>
+        <v>4.6466666666666665</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>13341</v>
+      </c>
+      <c r="B68">
+        <f t="shared" si="0"/>
+        <v>222.35</v>
+      </c>
+      <c r="C68">
+        <f t="shared" si="1"/>
+        <v>3.7058333333333335</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>20871</v>
+      </c>
+      <c r="B69">
+        <f t="shared" si="0"/>
+        <v>347.85</v>
+      </c>
+      <c r="C69">
+        <f t="shared" si="1"/>
+        <v>5.7975000000000003</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>29148</v>
+      </c>
+      <c r="B70">
+        <f t="shared" si="0"/>
+        <v>485.8</v>
+      </c>
+      <c r="C70">
+        <f t="shared" si="1"/>
+        <v>8.0966666666666658</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>19996</v>
+      </c>
+      <c r="B71">
+        <f t="shared" si="0"/>
+        <v>333.26666666666665</v>
+      </c>
+      <c r="C71">
+        <f t="shared" si="1"/>
+        <v>5.5544444444444441</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>21397</v>
+      </c>
+      <c r="B72">
+        <f t="shared" si="0"/>
+        <v>356.61666666666667</v>
+      </c>
+      <c r="C72">
+        <f t="shared" si="1"/>
+        <v>5.9436111111111112</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>19346</v>
+      </c>
+      <c r="B73">
+        <f t="shared" si="0"/>
+        <v>322.43333333333334</v>
+      </c>
+      <c r="C73">
+        <f t="shared" si="1"/>
+        <v>5.3738888888888887</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>24691</v>
+      </c>
+      <c r="B74">
+        <f t="shared" si="0"/>
+        <v>411.51666666666665</v>
+      </c>
+      <c r="C74">
+        <f t="shared" si="1"/>
+        <v>6.8586111111111112</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>20727</v>
+      </c>
+      <c r="B75">
+        <f t="shared" si="0"/>
+        <v>345.45</v>
+      </c>
+      <c r="C75">
+        <f t="shared" si="1"/>
+        <v>5.7575000000000003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>